<commit_message>
Edit Doc QC Fill in
</commit_message>
<xml_diff>
--- a/templates/Doc QC Template.xlsx
+++ b/templates/Doc QC Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Commercial Servicing\Document QC\BAKER HILL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFA417F-BCD4-465F-9BD9-EBB18FC94107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E26326-48C1-4485-90CE-2E682354C8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Sheet1" sheetId="6" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archive Checklist'!$A$10:$G$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archive Checklist'!$A$10:$G$164</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Archive Checklist'!$9:$10</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="231">
   <si>
     <t>Commercial Required Document Checklist</t>
   </si>
@@ -488,9 +488,6 @@
     <t>Business Asset Purchase Agreement - CML</t>
   </si>
   <si>
-    <t>Business Plans/Projections (Borrower) - CML</t>
-  </si>
-  <si>
     <t>Certificate of Title - CML</t>
   </si>
   <si>
@@ -906,6 +903,12 @@
   </si>
   <si>
     <t>Credit Review - Annual - CML</t>
+  </si>
+  <si>
+    <t>Environmental Indemnity Agreement - CML</t>
+  </si>
+  <si>
+    <t>Business Plan - CML</t>
   </si>
 </sst>
 </file>
@@ -1618,6 +1621,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1656,18 +1671,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2386,15 +2389,15 @@
       <c r="B44" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="D44" s="79"/>
-      <c r="E44" s="79"/>
+      <c r="D44" s="83"/>
+      <c r="E44" s="83"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B45" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="D45" s="79"/>
-      <c r="E45" s="79"/>
+      <c r="D45" s="83"/>
+      <c r="E45" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2420,7 +2423,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:M172"/>
+  <dimension ref="A1:M173"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -2434,16 +2437,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="36" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68" t="s">
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="69"/>
+      <c r="F1" s="73"/>
       <c r="G1" s="57"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2538,7 +2541,7 @@
         <v>53</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>53</v>
@@ -2574,7 +2577,7 @@
         <v>53</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D13" s="62" t="s">
         <v>53</v>
@@ -2604,7 +2607,7 @@
         <v>53</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>53</v>
@@ -2636,7 +2639,7 @@
         <v>53</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>53</v>
@@ -2681,7 +2684,7 @@
         <v>53</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>53</v>
@@ -2792,7 +2795,7 @@
         <v>53</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>53</v>
@@ -2869,7 +2872,7 @@
         <v>71</v>
       </c>
       <c r="C32" s="62" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D32" s="62" t="s">
         <v>78</v>
@@ -2884,7 +2887,7 @@
         <v>71</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>74</v>
@@ -2899,7 +2902,7 @@
         <v>71</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>74</v>
@@ -2916,7 +2919,7 @@
         <v>71</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>74</v>
@@ -2963,7 +2966,7 @@
         <v>71</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>78</v>
@@ -3006,7 +3009,7 @@
         <v>71</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>78</v>
@@ -3021,7 +3024,7 @@
         <v>71</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>78</v>
@@ -3053,10 +3056,10 @@
         <v>71</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E44" s="48"/>
       <c r="F44" s="10"/>
@@ -3128,7 +3131,7 @@
         <v>71</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>90</v>
+        <v>230</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>76</v>
@@ -3143,7 +3146,7 @@
         <v>71</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>78</v>
@@ -3158,7 +3161,7 @@
         <v>71</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>78</v>
@@ -3173,7 +3176,7 @@
         <v>71</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>86</v>
@@ -3188,7 +3191,7 @@
         <v>79</v>
       </c>
       <c r="C53" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" s="48"/>
@@ -3201,7 +3204,7 @@
         <v>71</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>78</v>
@@ -3216,7 +3219,7 @@
         <v>71</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>76</v>
@@ -3231,10 +3234,10 @@
         <v>71</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E56" s="48"/>
       <c r="F56" s="10"/>
@@ -3246,10 +3249,10 @@
         <v>71</v>
       </c>
       <c r="C57" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D57" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="E57" s="48"/>
       <c r="F57" s="10"/>
@@ -3261,7 +3264,7 @@
         <v>71</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>78</v>
@@ -3276,7 +3279,7 @@
         <v>71</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>78</v>
@@ -3291,10 +3294,10 @@
         <v>71</v>
       </c>
       <c r="C60" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D60" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="E60" s="48"/>
       <c r="F60" s="10"/>
@@ -3306,10 +3309,10 @@
         <v>71</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E61" s="48"/>
       <c r="F61" s="10"/>
@@ -3321,10 +3324,10 @@
         <v>71</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E62" s="48"/>
       <c r="F62" s="10"/>
@@ -3336,10 +3339,10 @@
         <v>71</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E63" s="48"/>
       <c r="F63" s="10"/>
@@ -3351,10 +3354,10 @@
         <v>71</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E64" s="48"/>
       <c r="F64" s="10"/>
@@ -3366,10 +3369,10 @@
         <v>71</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E65" s="48"/>
       <c r="F65" s="10"/>
@@ -3381,7 +3384,7 @@
         <v>71</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>78</v>
@@ -3396,10 +3399,10 @@
         <v>71</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E67" s="48"/>
       <c r="F67" s="10"/>
@@ -3411,10 +3414,10 @@
         <v>71</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E68" s="48"/>
       <c r="F68" s="10"/>
@@ -3426,10 +3429,10 @@
         <v>71</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E69" s="48"/>
       <c r="F69" s="10"/>
@@ -3441,7 +3444,7 @@
         <v>71</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>78</v>
@@ -3456,10 +3459,10 @@
         <v>71</v>
       </c>
       <c r="C71" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>110</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="E71" s="48"/>
       <c r="F71" s="10"/>
@@ -3471,7 +3474,7 @@
         <v>71</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>78</v>
@@ -3486,10 +3489,10 @@
         <v>71</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E73" s="48"/>
       <c r="F73" s="10"/>
@@ -3501,7 +3504,7 @@
         <v>71</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>76</v>
@@ -3515,13 +3518,13 @@
         <v>63</v>
       </c>
       <c r="B75" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C75" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C75" s="4" t="s">
-        <v>116</v>
-      </c>
       <c r="D75" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E75" s="48" t="s">
         <v>63</v>
@@ -3539,7 +3542,7 @@
         <v>71</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>76</v>
@@ -3551,10 +3554,10 @@
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="38"/>
       <c r="B77" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C77" s="31" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>53</v>
@@ -3569,10 +3572,10 @@
         <v>71</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E78" s="48"/>
       <c r="F78" s="10"/>
@@ -3584,10 +3587,10 @@
         <v>71</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E79" s="48"/>
       <c r="F79" s="10"/>
@@ -3599,7 +3602,7 @@
         <v>71</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>78</v>
@@ -3614,7 +3617,7 @@
         <v>71</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>78</v>
@@ -3626,13 +3629,13 @@
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="38"/>
       <c r="B82" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C82" s="4" t="s">
-        <v>121</v>
-      </c>
       <c r="D82" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E82" s="48"/>
       <c r="F82" s="10"/>
@@ -3641,10 +3644,10 @@
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="38"/>
       <c r="B83" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D83" s="1"/>
       <c r="E83" s="48"/>
@@ -3657,7 +3660,7 @@
         <v>71</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>78</v>
@@ -3672,7 +3675,7 @@
         <v>71</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>73</v>
@@ -3687,7 +3690,7 @@
         <v>71</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>78</v>
@@ -3702,7 +3705,7 @@
         <v>71</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>78</v>
@@ -3717,10 +3720,10 @@
         <v>71</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E88" s="48"/>
       <c r="F88" s="10"/>
@@ -3731,11 +3734,11 @@
       <c r="B89" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C89" s="4" t="s">
-        <v>200</v>
+      <c r="C89" s="10" t="s">
+        <v>229</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E89" s="48"/>
       <c r="F89" s="10"/>
@@ -3747,7 +3750,7 @@
         <v>71</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>128</v>
+        <v>199</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>74</v>
@@ -3762,10 +3765,10 @@
         <v>71</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E91" s="48"/>
       <c r="F91" s="10"/>
@@ -3777,7 +3780,7 @@
         <v>71</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>78</v>
@@ -3786,31 +3789,31 @@
       <c r="F92" s="10"/>
       <c r="G92" s="49"/>
     </row>
-    <row r="93" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="38"/>
       <c r="B93" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>210</v>
+        <v>129</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E93" s="48"/>
       <c r="F93" s="10"/>
       <c r="G93" s="49"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A94" s="38"/>
       <c r="B94" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E94" s="48"/>
       <c r="F94" s="10"/>
@@ -3822,10 +3825,10 @@
         <v>71</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>187</v>
+        <v>220</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E95" s="48"/>
       <c r="F95" s="10"/>
@@ -3837,44 +3840,44 @@
         <v>71</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E96" s="48"/>
       <c r="F96" s="10"/>
       <c r="G96" s="49"/>
     </row>
-    <row r="97" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="38"/>
       <c r="B97" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>132</v>
+        <v>184</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="E97" s="48"/>
       <c r="F97" s="10"/>
       <c r="G97" s="49"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A98" s="38"/>
       <c r="B98" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="E98" s="48"/>
       <c r="F98" s="10"/>
-      <c r="G98" s="58"/>
+      <c r="G98" s="49"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="38"/>
@@ -3882,10 +3885,10 @@
         <v>71</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>133</v>
+        <v>183</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E99" s="48"/>
       <c r="F99" s="10"/>
@@ -3897,14 +3900,14 @@
         <v>71</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="E100" s="48"/>
       <c r="F100" s="10"/>
-      <c r="G100" s="49"/>
+      <c r="G100" s="58"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="38"/>
@@ -3912,10 +3915,10 @@
         <v>71</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E101" s="48"/>
       <c r="F101" s="10"/>
@@ -3927,10 +3930,10 @@
         <v>71</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="E102" s="48"/>
       <c r="F102" s="10"/>
@@ -3942,10 +3945,10 @@
         <v>71</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E103" s="48"/>
       <c r="F103" s="10"/>
@@ -3957,7 +3960,7 @@
         <v>71</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>78</v>
@@ -3972,10 +3975,10 @@
         <v>71</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E105" s="48"/>
       <c r="F105" s="10"/>
@@ -3987,10 +3990,10 @@
         <v>71</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="E106" s="48"/>
       <c r="F106" s="10"/>
@@ -4002,10 +4005,10 @@
         <v>71</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="E107" s="48"/>
       <c r="F107" s="10"/>
@@ -4017,10 +4020,10 @@
         <v>71</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E108" s="48"/>
       <c r="F108" s="10"/>
@@ -4032,10 +4035,10 @@
         <v>71</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E109" s="48"/>
       <c r="F109" s="10"/>
@@ -4047,10 +4050,10 @@
         <v>71</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E110" s="48"/>
       <c r="F110" s="10"/>
@@ -4062,10 +4065,10 @@
         <v>71</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>189</v>
+        <v>144</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>78</v>
+        <v>141</v>
       </c>
       <c r="E111" s="48"/>
       <c r="F111" s="10"/>
@@ -4077,42 +4080,42 @@
         <v>71</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>146</v>
+        <v>188</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>147</v>
+        <v>78</v>
       </c>
       <c r="E112" s="48"/>
       <c r="F112" s="10"/>
       <c r="G112" s="49"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" s="38" t="s">
-        <v>63</v>
-      </c>
+      <c r="A113" s="38"/>
       <c r="B113" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E113" s="48"/>
       <c r="F113" s="10"/>
       <c r="G113" s="49"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" s="38"/>
+      <c r="A114" s="38" t="s">
+        <v>63</v>
+      </c>
       <c r="B114" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="E114" s="48"/>
       <c r="F114" s="10"/>
@@ -4124,7 +4127,7 @@
         <v>71</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D115" s="4" t="s">
         <v>78</v>
@@ -4139,7 +4142,7 @@
         <v>71</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>78</v>
@@ -4154,10 +4157,10 @@
         <v>71</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>222</v>
+        <v>151</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E117" s="48"/>
       <c r="F117" s="10"/>
@@ -4169,10 +4172,10 @@
         <v>71</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>153</v>
+        <v>221</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E118" s="48"/>
       <c r="F118" s="10"/>
@@ -4184,10 +4187,10 @@
         <v>71</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>192</v>
+        <v>152</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="E119" s="48"/>
       <c r="F119" s="10"/>
@@ -4199,40 +4202,40 @@
         <v>71</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>154</v>
+        <v>191</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>149</v>
+        <v>74</v>
       </c>
       <c r="E120" s="48"/>
       <c r="F120" s="10"/>
       <c r="G120" s="49"/>
     </row>
-    <row r="121" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="38"/>
       <c r="B121" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>76</v>
+        <v>148</v>
       </c>
       <c r="E121" s="48"/>
       <c r="F121" s="10"/>
       <c r="G121" s="49"/>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A122" s="38"/>
       <c r="B122" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>211</v>
+        <v>154</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E122" s="48"/>
       <c r="F122" s="10"/>
@@ -4244,7 +4247,7 @@
         <v>71</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>78</v>
@@ -4259,7 +4262,7 @@
         <v>71</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>156</v>
+        <v>196</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>78</v>
@@ -4269,14 +4272,12 @@
       <c r="G124" s="49"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A125" s="38" t="s">
-        <v>63</v>
-      </c>
+      <c r="A125" s="38"/>
       <c r="B125" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>78</v>
@@ -4286,15 +4287,17 @@
       <c r="G125" s="49"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" s="38"/>
+      <c r="A126" s="38" t="s">
+        <v>63</v>
+      </c>
       <c r="B126" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>216</v>
+        <v>156</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E126" s="48"/>
       <c r="F126" s="10"/>
@@ -4306,10 +4309,10 @@
         <v>71</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="E127" s="48"/>
       <c r="F127" s="10"/>
@@ -4321,7 +4324,7 @@
         <v>71</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>78</v>
@@ -4336,10 +4339,10 @@
         <v>71</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="E129" s="48"/>
       <c r="F129" s="10"/>
@@ -4351,10 +4354,10 @@
         <v>71</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E130" s="48"/>
       <c r="F130" s="10"/>
@@ -4366,7 +4369,7 @@
         <v>71</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>220</v>
+        <v>157</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>78</v>
@@ -4381,10 +4384,10 @@
         <v>71</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>159</v>
+        <v>219</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E132" s="48"/>
       <c r="F132" s="10"/>
@@ -4396,10 +4399,10 @@
         <v>71</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>226</v>
+        <v>158</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E133" s="48"/>
       <c r="F133" s="10"/>
@@ -4411,10 +4414,10 @@
         <v>71</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>160</v>
+        <v>225</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>149</v>
+        <v>78</v>
       </c>
       <c r="E134" s="48"/>
       <c r="F134" s="10"/>
@@ -4426,25 +4429,25 @@
         <v>71</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="E135" s="48"/>
       <c r="F135" s="10"/>
       <c r="G135" s="49"/>
     </row>
-    <row r="136" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="38"/>
       <c r="B136" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>227</v>
+        <v>160</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="E136" s="48"/>
       <c r="F136" s="10"/>
@@ -4456,25 +4459,25 @@
         <v>71</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D137" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E137" s="48"/>
       <c r="F137" s="10"/>
       <c r="G137" s="49"/>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A138" s="38"/>
       <c r="B138" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="E138" s="48"/>
       <c r="F138" s="10"/>
@@ -4486,10 +4489,10 @@
         <v>71</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="E139" s="48"/>
       <c r="F139" s="10"/>
@@ -4501,40 +4504,40 @@
         <v>71</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>162</v>
+        <v>205</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="E140" s="48"/>
       <c r="F140" s="10"/>
       <c r="G140" s="49"/>
     </row>
-    <row r="141" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="38"/>
       <c r="B141" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>201</v>
+        <v>161</v>
       </c>
       <c r="D141" s="4" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="E141" s="48"/>
       <c r="F141" s="10"/>
       <c r="G141" s="49"/>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A142" s="38"/>
       <c r="B142" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>78</v>
+        <v>130</v>
       </c>
       <c r="E142" s="48"/>
       <c r="F142" s="10"/>
@@ -4546,10 +4549,10 @@
         <v>71</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>163</v>
+        <v>222</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E143" s="48"/>
       <c r="F143" s="10"/>
@@ -4561,10 +4564,10 @@
         <v>71</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="E144" s="48"/>
       <c r="F144" s="10"/>
@@ -4576,7 +4579,7 @@
         <v>71</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>78</v>
@@ -4591,7 +4594,7 @@
         <v>71</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>213</v>
+        <v>164</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>78</v>
@@ -4606,7 +4609,7 @@
         <v>71</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>166</v>
+        <v>212</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>78</v>
@@ -4621,7 +4624,7 @@
         <v>71</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D148" s="4" t="s">
         <v>78</v>
@@ -4636,10 +4639,10 @@
         <v>71</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>224</v>
+        <v>166</v>
       </c>
       <c r="D149" s="4" t="s">
-        <v>149</v>
+        <v>78</v>
       </c>
       <c r="E149" s="48"/>
       <c r="F149" s="10"/>
@@ -4651,10 +4654,10 @@
         <v>71</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>168</v>
+        <v>223</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="E150" s="48"/>
       <c r="F150" s="10"/>
@@ -4666,7 +4669,7 @@
         <v>71</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>78</v>
@@ -4681,7 +4684,7 @@
         <v>71</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>78</v>
@@ -4696,7 +4699,7 @@
         <v>71</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>78</v>
@@ -4705,31 +4708,31 @@
       <c r="F153" s="10"/>
       <c r="G153" s="49"/>
     </row>
-    <row r="154" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="38"/>
       <c r="B154" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E154" s="48"/>
       <c r="F154" s="10"/>
       <c r="G154" s="49"/>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A155" s="38"/>
       <c r="B155" s="10" t="s">
         <v>71</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E155" s="48"/>
       <c r="F155" s="10"/>
@@ -4741,7 +4744,7 @@
         <v>71</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D156" s="4" t="s">
         <v>78</v>
@@ -4756,7 +4759,7 @@
         <v>71</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>78</v>
@@ -4766,142 +4769,157 @@
       <c r="G157" s="49"/>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A158" s="80"/>
-      <c r="B158" s="81" t="s">
-        <v>71</v>
-      </c>
-      <c r="C158" s="66" t="s">
-        <v>225</v>
-      </c>
-      <c r="D158" s="66" t="s">
+      <c r="A158" s="38"/>
+      <c r="B158" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D158" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E158" s="48"/>
+      <c r="F158" s="10"/>
+      <c r="G158" s="49"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" s="67"/>
+      <c r="B159" s="68" t="s">
+        <v>71</v>
+      </c>
+      <c r="C159" s="66" t="s">
+        <v>224</v>
+      </c>
+      <c r="D159" s="66" t="s">
         <v>83</v>
       </c>
-      <c r="E158" s="82"/>
-      <c r="F158" s="81"/>
-      <c r="G158" s="83"/>
-    </row>
-    <row r="159" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="39"/>
-      <c r="B159" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="C159" s="41" t="s">
+      <c r="E159" s="69"/>
+      <c r="F159" s="68"/>
+      <c r="G159" s="70"/>
+    </row>
+    <row r="160" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="39"/>
+      <c r="B160" s="40" t="s">
+        <v>71</v>
+      </c>
+      <c r="C160" s="41" t="s">
+        <v>175</v>
+      </c>
+      <c r="D160" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="E160" s="50"/>
+      <c r="F160" s="40"/>
+      <c r="G160" s="51"/>
+    </row>
+    <row r="162" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="1">
+        <f>SUM(A11:A30)</f>
+        <v>0</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C162" s="2"/>
+      <c r="D162" s="2"/>
+      <c r="E162" s="55">
+        <f>SUM(E12:E160)</f>
+        <v>0</v>
+      </c>
+      <c r="F162" s="1"/>
+      <c r="G162" s="1"/>
+    </row>
+    <row r="163" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="1">
+        <f>SUM(A31:A160)</f>
+        <v>0</v>
+      </c>
+      <c r="B163" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D159" s="41" t="s">
-        <v>78</v>
-      </c>
-      <c r="E159" s="50"/>
-      <c r="F159" s="40"/>
-      <c r="G159" s="51"/>
-    </row>
-    <row r="161" spans="1:7" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="1">
-        <f>SUM(A12:A30)</f>
+      <c r="C163" s="1"/>
+    </row>
+    <row r="164" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="43">
+        <f>SUM(A162:A163)</f>
         <v>0</v>
       </c>
-      <c r="B161" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C161" s="2"/>
-      <c r="D161" s="2"/>
-      <c r="E161" s="55">
-        <f>SUM(E12:E159)</f>
-        <v>0</v>
-      </c>
-      <c r="F161" s="1"/>
-      <c r="G161" s="1"/>
-    </row>
-    <row r="162" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="1">
-        <f>SUM(A31:A159)</f>
-        <v>0</v>
-      </c>
-      <c r="B162" s="1" t="s">
+      <c r="B164" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C162" s="1"/>
-    </row>
-    <row r="163" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="43">
-        <f>SUM(A161:A162)</f>
-        <v>0</v>
-      </c>
-      <c r="B163" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="C163" s="1"/>
-    </row>
-    <row r="164" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A164" s="29"/>
-      <c r="B164" s="29"/>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B165" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C165" s="8"/>
+      <c r="C164" s="1"/>
+    </row>
+    <row r="165" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A165" s="29"/>
+      <c r="B165" s="29"/>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B166" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="C166" s="9"/>
-    </row>
-    <row r="167" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B168" s="70"/>
-      <c r="C168" s="71"/>
-      <c r="D168" s="71"/>
-      <c r="E168" s="71"/>
-      <c r="F168" s="71"/>
-      <c r="G168" s="72"/>
-    </row>
+        <v>178</v>
+      </c>
+      <c r="C166" s="8"/>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B167" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B169" s="73"/>
-      <c r="C169" s="74"/>
-      <c r="D169" s="74"/>
-      <c r="E169" s="74"/>
-      <c r="F169" s="74"/>
-      <c r="G169" s="75"/>
+      <c r="B169" s="74"/>
+      <c r="C169" s="75"/>
+      <c r="D169" s="75"/>
+      <c r="E169" s="75"/>
+      <c r="F169" s="75"/>
+      <c r="G169" s="76"/>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B170" s="73"/>
-      <c r="C170" s="74"/>
-      <c r="D170" s="74"/>
-      <c r="E170" s="74"/>
-      <c r="F170" s="74"/>
-      <c r="G170" s="75"/>
+      <c r="B170" s="77"/>
+      <c r="C170" s="78"/>
+      <c r="D170" s="78"/>
+      <c r="E170" s="78"/>
+      <c r="F170" s="78"/>
+      <c r="G170" s="79"/>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B171" s="73"/>
-      <c r="C171" s="74"/>
-      <c r="D171" s="74"/>
-      <c r="E171" s="74"/>
-      <c r="F171" s="74"/>
-      <c r="G171" s="75"/>
-    </row>
-    <row r="172" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B172" s="76"/>
-      <c r="C172" s="77"/>
-      <c r="D172" s="77"/>
-      <c r="E172" s="77"/>
-      <c r="F172" s="77"/>
-      <c r="G172" s="78"/>
+      <c r="B171" s="77"/>
+      <c r="C171" s="78"/>
+      <c r="D171" s="78"/>
+      <c r="E171" s="78"/>
+      <c r="F171" s="78"/>
+      <c r="G171" s="79"/>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B172" s="77"/>
+      <c r="C172" s="78"/>
+      <c r="D172" s="78"/>
+      <c r="E172" s="78"/>
+      <c r="F172" s="78"/>
+      <c r="G172" s="79"/>
+    </row>
+    <row r="173" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B173" s="80"/>
+      <c r="C173" s="81"/>
+      <c r="D173" s="81"/>
+      <c r="E173" s="81"/>
+      <c r="F173" s="81"/>
+      <c r="G173" s="82"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:G163" xr:uid="{00000000-0001-0000-0300-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A31:G163">
-      <sortCondition ref="C10:C163"/>
+  <autoFilter ref="A10:G164" xr:uid="{00000000-0001-0000-0300-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A31:G164">
+      <sortCondition ref="C10:C164"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A31:G160">
-    <sortCondition ref="C31:C160"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A31:G161">
+    <sortCondition ref="C31:C161"/>
   </sortState>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="B168:G172"/>
+    <mergeCell ref="B169:G173"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="74" orientation="portrait" verticalDpi="300" r:id="rId1"/>
@@ -4988,12 +5006,12 @@
   <sheetData>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -5002,21 +5020,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010029B669A0FB19994B974F97D314543741" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8f00360ad354c32f6313117303b768de">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0b0e1ac4-03a7-4459-80ca-b68e6c422d22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f81d7e9f0a47e375a96a9e4e03a4ff17" ns3:_="">
     <xsd:import namespace="0b0e1ac4-03a7-4459-80ca-b68e6c422d22"/>
@@ -5180,15 +5189,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C5408DE-558F-4B7A-B26F-9474AA13BABB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3225117-15A9-437C-AA70-4BDC9D1F6FD4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5197,7 +5207,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D4E762B-AD05-456C-98E6-BE2D50F536DC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5213,4 +5223,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C5408DE-558F-4B7A-B26F-9474AA13BABB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>